<commit_message>
🔄 [Automazione] Aggiornamento anagrafica locali tramite incrocio AWP GamesLodi
</commit_message>
<xml_diff>
--- a/elenco_locali.xlsx
+++ b/elenco_locali.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C164"/>
+  <dimension ref="A1:C165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -633,7 +633,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>NTS Networks</t>
+          <t>Snaitech Spa WG</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Snaitech Spa WG</t>
+          <t>NTS Networks</t>
         </is>
       </c>
     </row>
@@ -2918,29 +2918,29 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>EA110058135S</t>
+          <t>EA670043281S</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>TABACCHERIA ORCHIDEA VERDE</t>
+          <t>TABACCHERIA N. 10_NTS</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Snaitech Spa WG</t>
+          <t>NTS Networks</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>EA590017319S</t>
+          <t>EA110058135S</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>TABACCHERIA RICEVITORIA VISENTINI PAOLO</t>
+          <t>TABACCHERIA ORCHIDEA VERDE</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -2952,12 +2952,12 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>EA670026114S</t>
+          <t>EA590017319S</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>TABACCHERIA ROSTAGNO</t>
+          <t>TABACCHERIA RICEVITORIA VISENTINI PAOLO</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -2969,12 +2969,12 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>EA570132577S</t>
+          <t>EA670026114S</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>TABACCHERIA THE BLACK CROW DI PELLICANO' ROBERTO</t>
+          <t>TABACCHERIA ROSTAGNO</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -2986,12 +2986,12 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>EA910070191J</t>
+          <t>EA570132577S</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>TABACCHERIA VENETA DI PALMA ALESSANDRA</t>
+          <t>TABACCHERIA THE BLACK CROW DI PELLICANO' ROBERTO</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -3003,12 +3003,12 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>EA110057947A</t>
+          <t>EA910070191J</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>TABACCHI DELLA PIAZZA DI LIN ELENA</t>
+          <t>TABACCHERIA VENETA DI PALMA ALESSANDRA</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -3020,12 +3020,12 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>EA110043088F</t>
+          <t>EA110057947A</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>TABACCHI DI CHEN MAOXI</t>
+          <t>TABACCHI DELLA PIAZZA DI LIN ELENA</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -3037,12 +3037,12 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>EA230203099S</t>
+          <t>EA110043088F</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>TABACCHI EDICOLA RIV. N.6</t>
+          <t>TABACCHI DI CHEN MAOXI</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -3054,12 +3054,12 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>EA230014587S</t>
+          <t>EA230203099S</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>TABACCHI FRANZOI</t>
+          <t>TABACCHI EDICOLA RIV. N.6</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -3071,46 +3071,46 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>EA750215537S</t>
+          <t>EA230014587S</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>TABACCHI PITZALIS</t>
+          <t>TABACCHI FRANZOI</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>NTS Networks</t>
+          <t>Snaitech Spa WG</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>EA570075631A</t>
+          <t>EA750215537S</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>TAVERNA DEL LUFF</t>
+          <t>TABACCHI PITZALIS</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Snaitech Spa WG</t>
+          <t>NTS Networks</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>EA560080343Y</t>
+          <t>EA570075631A</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>TOFE' CAFE'</t>
+          <t>TAVERNA DEL LUFF</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -3122,12 +3122,12 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>EA570011433R</t>
+          <t>EA560080343Y</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>ULTIMA PRIMA BAR TABACCHI</t>
+          <t>TOFE' CAFE'</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -3144,61 +3144,78 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>ULTIMA PRIMA BAR TABACCHI - SERVICE</t>
+          <t>ULTIMA PRIMA BAR TABACCHI</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>SNAITECH SPA</t>
+          <t>Snaitech Spa WG</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>EA740113636H</t>
+          <t>EA570011433R</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>VILLAURBANA.NET</t>
+          <t>ULTIMA PRIMA BAR TABACCHI - SERVICE</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>NTS Networks</t>
+          <t>SNAITECH SPA</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>EA110061648W</t>
+          <t>EA740113636H</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>WG TABACCHERIA CHIAPPETTA DEBORA</t>
+          <t>VILLAURBANA.NET</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Snaitech Spa WG</t>
+          <t>NTS Networks</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
+          <t>EA110061648W</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>WG TABACCHERIA CHIAPPETTA DEBORA</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Snaitech Spa WG</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
           <t>EA110213491R</t>
         </is>
       </c>
-      <c r="B164" t="inlineStr">
+      <c r="B165" t="inlineStr">
         <is>
           <t>WINNER CAFFE'</t>
         </is>
       </c>
-      <c r="C164" t="inlineStr">
+      <c r="C165" t="inlineStr">
         <is>
           <t>Snaitech Spa WG</t>
         </is>

</xml_diff>